<commit_message>
chore: clean up store code and sync product schema
- Remove the unused AI chatbot feature
- Remove old test data, demo files, seed files, and unused scripts
- Clean up unused Store Manager code
- Remove the product unit feature from backend and frontend
- Add a safe migration to sync the product schema with the database
</commit_message>
<xml_diff>
--- a/client/public/import_template.xlsx
+++ b/client/public/import_template.xlsx
@@ -4,8 +4,87 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Sản phẩm nhập" sheetId="1" r:id="rId1"/>
+    <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Sản phẩm nhập'!A1:M1</definedName>
+  </definedNames>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>PetMatching</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <t>Để trống để hệ thống tự tạo mã. Dùng mã hiện có khi muốn cập nhật sản phẩm.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0">
+      <text>
+        <t>Tên sản phẩm; với nhiều phân loại, lặp lại cùng tên trên từng dòng.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <t>Tên biến thể như Size M hoặc Hộp 500g. Mỗi phân loại dùng một dòng.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0">
+      <text>
+        <t>Tên danh mục. Hệ thống tự chuẩn hóa và tạo danh mục chưa tồn tại.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
+      <text>
+        <t>Tên thương hiệu sản phẩm.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
+      <text>
+        <t>Ví dụ: cái, túi, hộp, chai.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0">
+      <text>
+        <t>Số lớn hơn 0 và không được lớn hơn Giá bán.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0">
+      <text>
+        <t>Số lớn hơn 0.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <t>Để trống nếu không áp dụng khuyến mãi.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <t>Số từ 0 trở lên; để trống được hiểu là 0.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <t>Chỉ dùng DOG, CAT hoặc ALL; để trống được hiểu là ALL.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0">
+      <text>
+        <t>Dạng Thuộc tính: Giá trị, Thuộc tính 2: Giá trị 2.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0">
+      <text>
+        <t>Mô tả ngắn gọn về sản phẩm.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
@@ -397,9 +476,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M1"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="44.83203125" customWidth="1"/>
+    <col min="13" max="13" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" t="str">
         <v>Mã sản phẩm</v>
       </c>
@@ -407,115 +501,258 @@
         <v>Tên sản phẩm</v>
       </c>
       <c r="C1" t="str">
+        <v>Phân loại</v>
+      </c>
+      <c r="D1" t="str">
         <v>Danh mục</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Thương hiệu</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Đơn vị tính</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Giá nhập</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Giá bán</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Giá khuyến mãi</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Số lượng nhập</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Loài mục tiêu</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Thông số kỹ thuật</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Mô tả</v>
       </c>
     </row>
-    <row r="2">
+  </sheetData>
+  <autoFilter ref="A1:M1"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+  </ignoredErrors>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C22"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="88.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" t="str">
+        <v>HƯỚNG DẪN IMPORT SẢN PHẨM</v>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
       <c r="A2" t="str">
-        <v>128222</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Luoc chai long tu dong cho thu cung</v>
-      </c>
-      <c r="C2" t="str">
-        <v>GROOMING</v>
-      </c>
-      <c r="D2" t="str">
-        <v>FurCare</v>
-      </c>
-      <c r="E2" t="str">
-        <v>cái</v>
-      </c>
-      <c r="F2">
-        <v>60000</v>
-      </c>
-      <c r="G2">
-        <v>135000</v>
-      </c>
-      <c r="H2">
-        <v>109000</v>
-      </c>
-      <c r="I2">
-        <v>10</v>
-      </c>
-      <c r="J2" t="str">
-        <v>ALL</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Màu sắc: Hồng, Kích thước: Trung bình, Chất liệu: Nhựa &amp; Thép</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Lược chải lông tự động cho chó mèo.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>999999</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Sản phẩm thử nghiệm mới Excel</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ACCESSORY</v>
-      </c>
-      <c r="D3" t="str">
-        <v>PetBrand</v>
-      </c>
-      <c r="E3" t="str">
-        <v>cái</v>
-      </c>
-      <c r="F3">
-        <v>50000</v>
-      </c>
-      <c r="G3">
-        <v>100000</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3">
-        <v>20</v>
-      </c>
-      <c r="J3" t="str">
-        <v>CAT</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Chất liệu: Cotton, Độ bền: Cao</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Sản phẩm test tạo mới hoàn toàn từ file Excel.</v>
+        <v>Nhập dữ liệu tại sheet “Sản phẩm nhập”. Không đổi tên các cột.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Cột</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Bắt buộc</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Quy tắc nhập</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Mã sản phẩm</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Để trống để hệ thống tự tạo mã. Dùng mã hiện có khi muốn cập nhật sản phẩm.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tên sản phẩm</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Có</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Tên sản phẩm; với nhiều phân loại, lặp lại cùng tên trên từng dòng.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Phân loại</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Tên biến thể như Size M hoặc Hộp 500g. Mỗi phân loại dùng một dòng.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Danh mục</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Có</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Tên danh mục. Hệ thống tự chuẩn hóa và tạo danh mục chưa tồn tại.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Thương hiệu</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Tên thương hiệu sản phẩm.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Đơn vị tính</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Ví dụ: cái, túi, hộp, chai.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Giá nhập</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Có</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Số lớn hơn 0 và không được lớn hơn Giá bán.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Giá bán</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Có</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Số lớn hơn 0.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Giá khuyến mãi</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Để trống nếu không áp dụng khuyến mãi.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Số lượng nhập</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Số từ 0 trở lên; để trống được hiểu là 0.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Loài mục tiêu</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Chỉ dùng DOG, CAT hoặc ALL; để trống được hiểu là ALL.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Thông số kỹ thuật</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Dạng Thuộc tính: Giá trị, Thuộc tính 2: Giá trị 2.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Mô tả</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Mô tả ngắn gọn về sản phẩm.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Ảnh sản phẩm</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Ảnh chính</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Đặt trong thư mục có tên trùng Mã sản phẩm, hoặc đặt tên file bắt đầu bằng Mã sản phẩm.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Ảnh phân loại</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Dùng thư mục/tên file theo dạng Mã sản phẩm-Phân loại hoặc Mã sản phẩm_Phân loại.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Lưu ý</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Khi import, hệ thống cộng “Số lượng nhập” vào tồn kho hiện tại thay vì thay thế tồn kho.</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A19:C19"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(manager): cap nhat dong bo trang thai mo ban giua san pham va variant, toi uu phi ship va xu ly don hang
</commit_message>
<xml_diff>
--- a/client/public/import_template.xlsx
+++ b/client/public/import_template.xlsx
@@ -6,85 +6,7 @@
     <sheet name="Sản phẩm nhập" sheetId="1" r:id="rId1"/>
     <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Sản phẩm nhập'!A1:M1</definedName>
-  </definedNames>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>PetMatching</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0">
-      <text>
-        <t>Để trống để hệ thống tự tạo mã. Dùng mã hiện có khi muốn cập nhật sản phẩm.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0">
-      <text>
-        <t>Tên sản phẩm; với nhiều phân loại, lặp lại cùng tên trên từng dòng.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0">
-      <text>
-        <t>Tên biến thể như Size M hoặc Hộp 500g. Mỗi phân loại dùng một dòng.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0">
-      <text>
-        <t>Tên danh mục. Hệ thống tự chuẩn hóa và tạo danh mục chưa tồn tại.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0">
-      <text>
-        <t>Tên thương hiệu sản phẩm.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0">
-      <text>
-        <t>Ví dụ: cái, túi, hộp, chai.</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0">
-      <text>
-        <t>Số lớn hơn 0 và không được lớn hơn Giá bán.</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0">
-      <text>
-        <t>Số lớn hơn 0.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0">
-      <text>
-        <t>Để trống nếu không áp dụng khuyến mãi.</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0">
-      <text>
-        <t>Số từ 0 trở lên; để trống được hiểu là 0.</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0">
-      <text>
-        <t>Chỉ dùng DOG, CAT hoặc ALL; để trống được hiểu là ALL.</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0">
-      <text>
-        <t>Dạng Thuộc tính: Giá trị, Thuộc tính 2: Giá trị 2.</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0">
-      <text>
-        <t>Mô tả ngắn gọn về sản phẩm.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
@@ -476,24 +398,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="44.83203125" customWidth="1"/>
-    <col min="13" max="13" width="48.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="35.83203125" customWidth="1"/>
+    <col min="13" max="13" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" t="str">
         <v>Mã sản phẩm</v>
       </c>
@@ -534,225 +456,332 @@
         <v>Mô tả</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>PROD_001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Thức ăn Hạt Hỗn Hợp Cho Chó Vị Bò</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Túi 1.5kg</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Thức ăn cho chó</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Pedigree</v>
+      </c>
+      <c r="F2" t="str">
+        <v>túi</v>
+      </c>
+      <c r="G2">
+        <v>120000</v>
+      </c>
+      <c r="H2">
+        <v>180000</v>
+      </c>
+      <c r="I2">
+        <v>159000</v>
+      </c>
+      <c r="J2">
+        <v>20</v>
+      </c>
+      <c r="K2" t="str">
+        <v>DOG</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Trọng lượng: 1.5kg, Xuất xứ: Thái Lan</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Thức ăn hạt dinh dưỡng cân bằng dành cho chó trưởng thành.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>PROD_001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Thức ăn Hạt Hỗn Hợp Cho Chó Vị Bò</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Túi 5kg</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Thức ăn cho chó</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Pedigree</v>
+      </c>
+      <c r="F3" t="str">
+        <v>túi</v>
+      </c>
+      <c r="G3">
+        <v>350000</v>
+      </c>
+      <c r="H3">
+        <v>500000</v>
+      </c>
+      <c r="I3">
+        <v>449000</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
+      </c>
+      <c r="K3" t="str">
+        <v>DOG</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Trọng lượng: 5kg, Xuất xứ: Thái Lan</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Thức ăn hạt dinh dưỡng cân bằng dành cho chó trưởng thành.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v>Pate Mèo Vị Cá Hồi Cấp Ẩm</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Hộp 400g</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Thức ăn cho mèo</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Whiskas</v>
+      </c>
+      <c r="F4" t="str">
+        <v>hộp</v>
+      </c>
+      <c r="G4">
+        <v>25000</v>
+      </c>
+      <c r="H4">
+        <v>45000</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4">
+        <v>50</v>
+      </c>
+      <c r="K4" t="str">
+        <v>CAT</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Khối lượng: 400g, Dạng: Pate</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Pate tươi thơm ngon giúp cấp nước và bổ sung vi chất cho mèo.</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M1"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C21"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="88.83203125" customWidth="1"/>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="80.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" t="str">
-        <v>HƯỚNG DẪN IMPORT SẢN PHẨM</v>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
+        <v>HƯỚNG DẪN IMPORT SẢN PHẨM &amp; TỒN KHO</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="str">
-        <v>Nhập dữ liệu tại sheet “Sản phẩm nhập”. Không đổi tên các cột.</v>
+        <v>1. Nhập dữ liệu tại sheet "Sản phẩm nhập". Giữ nguyên tiêu đề cột.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2. CẬP NHẬT TỒN KHO &amp; THÔNG TIN: Nếu nhập Mã sản phẩm (ví dụ: PROD_001) hoặc Tên sản phẩm đã có, hệ thống sẽ CẬP NHẬT thông tin và CỘNG DỒN số lượng nhập vào tồn kho.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Cột</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Bắt buộc</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Quy tắc nhập</v>
+        <v>3. THÊM SẢN PHẨM MỚI: Nếu để trống Mã sản phẩm và Tên sản phẩm chưa có trong hệ thống, hệ thống sẽ TỰ TẠO SẢN PHẨM MỚI.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Mã sản phẩm</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Để trống để hệ thống tự tạo mã. Dùng mã hiện có khi muốn cập nhật sản phẩm.</v>
+        <v>4. NHIỀU PHÂN LOẠI (VARIANT): Mỗi phân loại dùng 1 dòng, giữ nguyên Tên sản phẩm và Mã sản phẩm (nếu có).</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Tên sản phẩm</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Có</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Tên sản phẩm; với nhiều phân loại, lặp lại cùng tên trên từng dòng.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Phân loại</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Tên biến thể như Size M hoặc Hộp 500g. Mỗi phân loại dùng một dòng.</v>
+        <v>5. NHẬP KÈM ẢNH BẰNG THƯ MỤC: Đặt file Excel vào thư mục gốc. Tạo các thư mục con có tên là Mã sản phẩm (VD: PROD_001) hoặc Mã_Sản_Phẩm-Tên_Phân_Loại (VD: PROD_001-Túi 1.5kg) chứa file ảnh (.jpg, .png).</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Danh mục</v>
+        <v>Cột</v>
       </c>
       <c r="B8" t="str">
-        <v>Có</v>
+        <v>Bắt buộc</v>
       </c>
       <c r="C8" t="str">
-        <v>Tên danh mục. Hệ thống tự chuẩn hóa và tạo danh mục chưa tồn tại.</v>
+        <v>Quy tắc nhập</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Thương hiệu</v>
+        <v>Mã sản phẩm</v>
       </c>
       <c r="B9" t="str">
         <v>Không</v>
       </c>
       <c r="C9" t="str">
-        <v>Tên thương hiệu sản phẩm.</v>
+        <v>Nếu cập nhật sản phẩm cũ hãy điền Mã sản phẩm. Nếu tạo mới có thể để trống.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Đơn vị tính</v>
+        <v>Tên sản phẩm</v>
       </c>
       <c r="B10" t="str">
-        <v>Không</v>
+        <v>Có</v>
       </c>
       <c r="C10" t="str">
-        <v>Ví dụ: cái, túi, hộp, chai.</v>
+        <v>Tên sản phẩm. Với sản phẩm nhiều phân loại, điền cùng tên sản phẩm trên các dòng.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Giá nhập</v>
+        <v>Phân loại</v>
       </c>
       <c r="B11" t="str">
-        <v>Có</v>
+        <v>Không</v>
       </c>
       <c r="C11" t="str">
-        <v>Số lớn hơn 0 và không được lớn hơn Giá bán.</v>
+        <v>Tên phân loại/biến thể (VD: Túi 1.5kg, Hộp 400g, Size L, Màu Đỏ).</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Giá bán</v>
+        <v>Danh mục</v>
       </c>
       <c r="B12" t="str">
         <v>Có</v>
       </c>
       <c r="C12" t="str">
-        <v>Số lớn hơn 0.</v>
+        <v>Danh mục sản phẩm (VD: Thức ăn cho chó, Thức ăn cho mèo, Phụ kiện thú cưng).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Giá khuyến mãi</v>
+        <v>Thương hiệu</v>
       </c>
       <c r="B13" t="str">
         <v>Không</v>
       </c>
       <c r="C13" t="str">
-        <v>Để trống nếu không áp dụng khuyến mãi.</v>
+        <v>Tên thương hiệu sản phẩm (VD: Pedigree, Whiskas, Royal Canin).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Số lượng nhập</v>
+        <v>Đơn vị tính</v>
       </c>
       <c r="B14" t="str">
         <v>Không</v>
       </c>
       <c r="C14" t="str">
-        <v>Số từ 0 trở lên; để trống được hiểu là 0.</v>
+        <v>Ví dụ: túi, hộp, cái, lon, chai.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Loài mục tiêu</v>
+        <v>Giá nhập</v>
       </c>
       <c r="B15" t="str">
-        <v>Không</v>
+        <v>Có</v>
       </c>
       <c r="C15" t="str">
-        <v>Chỉ dùng DOG, CAT hoặc ALL; để trống được hiểu là ALL.</v>
+        <v>Giá nhập hàng (Số &gt; 0, &lt;= Giá bán).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Thông số kỹ thuật</v>
+        <v>Giá bán</v>
       </c>
       <c r="B16" t="str">
-        <v>Không</v>
+        <v>Có</v>
       </c>
       <c r="C16" t="str">
-        <v>Dạng Thuộc tính: Giá trị, Thuộc tính 2: Giá trị 2.</v>
+        <v>Giá bán niêm yết (Số &gt; 0).</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Mô tả</v>
+        <v>Giá khuyến mãi</v>
       </c>
       <c r="B17" t="str">
         <v>Không</v>
       </c>
       <c r="C17" t="str">
-        <v>Mô tả ngắn gọn về sản phẩm.</v>
+        <v>Giá khuyến mãi (để trống nếu không giảm giá).</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Số lượng nhập</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Số lượng nhập thêm vào kho (Số &gt;= 0).</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Ảnh sản phẩm</v>
+        <v>Loài mục tiêu</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Không</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Điền DOG (Cho chó), CAT (Cho mèo), hoặc ALL (Mọi thú cưng).</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Ảnh chính</v>
+        <v>Thông số kỹ thuật</v>
       </c>
       <c r="B20" t="str">
-        <v>Đặt trong thư mục có tên trùng Mã sản phẩm, hoặc đặt tên file bắt đầu bằng Mã sản phẩm.</v>
+        <v>Không</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Định dạng dạng: Thuộc tính 1: Giá trị 1, Thuộc tính 2: Giá trị 2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Ảnh phân loại</v>
+        <v>Mô tả</v>
       </c>
       <c r="B21" t="str">
-        <v>Dùng thư mục/tên file theo dạng Mã sản phẩm-Phân loại hoặc Mã sản phẩm_Phân loại.</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Lưu ý</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Khi import, hệ thống cộng “Số lượng nhập” vào tồn kho hiện tại thay vì thay thế tồn kho.</v>
+        <v>Không</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Mô tả chi tiết sản phẩm.</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A19:C19"/>
-  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(shop): sync order address calculation, optimize excel import template and cleanup manager UI
</commit_message>
<xml_diff>
--- a/client/public/import_template.xlsx
+++ b/client/public/import_template.xlsx
@@ -3,8 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sản phẩm nhập" sheetId="1" r:id="rId1"/>
-    <sheet name="Hướng dẫn" sheetId="2" r:id="rId2"/>
+    <sheet name="ImportTemplate" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -399,21 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M4"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="35.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
-    <col min="12" max="12" width="35.83203125" customWidth="1"/>
-    <col min="13" max="13" width="50.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,7 +416,7 @@
         <v>Thương hiệu</v>
       </c>
       <c r="F1" t="str">
-        <v>Đơn vị tính</v>
+        <v>Trọng lượng (kg)</v>
       </c>
       <c r="G1" t="str">
         <v>Giá nhập</v>
@@ -472,8 +456,8 @@
       <c r="E2" t="str">
         <v>Pedigree</v>
       </c>
-      <c r="F2" t="str">
-        <v>túi</v>
+      <c r="F2">
+        <v>1.5</v>
       </c>
       <c r="G2">
         <v>120000</v>
@@ -513,8 +497,8 @@
       <c r="E3" t="str">
         <v>Pedigree</v>
       </c>
-      <c r="F3" t="str">
-        <v>túi</v>
+      <c r="F3">
+        <v>5</v>
       </c>
       <c r="G3">
         <v>350000</v>
@@ -554,8 +538,8 @@
       <c r="E4" t="str">
         <v>Whiskas</v>
       </c>
-      <c r="F4" t="str">
-        <v>hộp</v>
+      <c r="F4">
+        <v>0.4</v>
       </c>
       <c r="G4">
         <v>25000</v>
@@ -584,204 +568,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>HƯỚNG DẪN IMPORT SẢN PHẨM &amp; TỒN KHO</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>1. Nhập dữ liệu tại sheet "Sản phẩm nhập". Giữ nguyên tiêu đề cột.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>2. CẬP NHẬT TỒN KHO &amp; THÔNG TIN: Nếu nhập Mã sản phẩm (ví dụ: PROD_001) hoặc Tên sản phẩm đã có, hệ thống sẽ CẬP NHẬT thông tin và CỘNG DỒN số lượng nhập vào tồn kho.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>3. THÊM SẢN PHẨM MỚI: Nếu để trống Mã sản phẩm và Tên sản phẩm chưa có trong hệ thống, hệ thống sẽ TỰ TẠO SẢN PHẨM MỚI.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>4. NHIỀU PHÂN LOẠI (VARIANT): Mỗi phân loại dùng 1 dòng, giữ nguyên Tên sản phẩm và Mã sản phẩm (nếu có).</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>5. NHẬP KÈM ẢNH BẰNG THƯ MỤC: Đặt file Excel vào thư mục gốc. Tạo các thư mục con có tên là Mã sản phẩm (VD: PROD_001) hoặc Mã_Sản_Phẩm-Tên_Phân_Loại (VD: PROD_001-Túi 1.5kg) chứa file ảnh (.jpg, .png).</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Cột</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Bắt buộc</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Quy tắc nhập</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Mã sản phẩm</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Nếu cập nhật sản phẩm cũ hãy điền Mã sản phẩm. Nếu tạo mới có thể để trống.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Tên sản phẩm</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Có</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Tên sản phẩm. Với sản phẩm nhiều phân loại, điền cùng tên sản phẩm trên các dòng.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Phân loại</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Tên phân loại/biến thể (VD: Túi 1.5kg, Hộp 400g, Size L, Màu Đỏ).</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Danh mục</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Có</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Danh mục sản phẩm (VD: Thức ăn cho chó, Thức ăn cho mèo, Phụ kiện thú cưng).</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Thương hiệu</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Tên thương hiệu sản phẩm (VD: Pedigree, Whiskas, Royal Canin).</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Đơn vị tính</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Ví dụ: túi, hộp, cái, lon, chai.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Giá nhập</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Có</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Giá nhập hàng (Số &gt; 0, &lt;= Giá bán).</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Giá bán</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Có</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Giá bán niêm yết (Số &gt; 0).</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Giá khuyến mãi</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Giá khuyến mãi (để trống nếu không giảm giá).</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Số lượng nhập</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Số lượng nhập thêm vào kho (Số &gt;= 0).</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Loài mục tiêu</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C19" t="str">
-        <v>Điền DOG (Cho chó), CAT (Cho mèo), hoặc ALL (Mọi thú cưng).</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Thông số kỹ thuật</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Định dạng dạng: Thuộc tính 1: Giá trị 1, Thuộc tính 2: Giá trị 2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Mô tả</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Không</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Mô tả chi tiết sản phẩm.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C21"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>